<commit_message>
Loads of new counters, map, cards, rules
Signed-off-by: euroledger <geominat@gmail.com>
</commit_message>
<xml_diff>
--- a/Cards_Fuhrer.xlsx
+++ b/Cards_Fuhrer.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\StateOfSiege Normandy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC69CD93-AC3E-49EF-B81A-4BDD0CAA300F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C2D2742-462B-48DB-BB5E-4FC448ACD167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="138">
   <si>
     <t>Starting Position</t>
   </si>
@@ -250,9 +250,6 @@
     <t>Operation Cobra</t>
   </si>
   <si>
-    <t>CALCULATE VICTORY: If Caen, Cherbourg and Avranches all lost - LOSE GAME.</t>
-  </si>
-  <si>
     <t>26</t>
   </si>
   <si>
@@ -409,46 +406,37 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>2 US; 1 Reinf</t>
-  </si>
-  <si>
-    <t>2 GB 1 Corps; 1 Supply</t>
-  </si>
-  <si>
-    <t>2 Reinf; 1 Supply</t>
-  </si>
-  <si>
     <t>3 US</t>
   </si>
   <si>
-    <t>3 Supply</t>
-  </si>
-  <si>
     <t>3 GB 1 Corps</t>
   </si>
   <si>
-    <t>3 Reinf</t>
-  </si>
-  <si>
     <t xml:space="preserve">3 GB </t>
   </si>
   <si>
     <t>1 US; 1 GB 2; 1 GB 1 Corps</t>
   </si>
   <si>
-    <t>1 GB 2; 1 GB 1 Corps;1 Reinf</t>
-  </si>
-  <si>
     <t xml:space="preserve">3 GB2 </t>
   </si>
   <si>
     <t>3 GB1 Corps</t>
   </si>
   <si>
-    <t>2 Supply; 1 Reinf</t>
-  </si>
-  <si>
-    <t>2 US; 1 Supply</t>
+    <t>2 US</t>
+  </si>
+  <si>
+    <t>2 GB 1 Corps</t>
+  </si>
+  <si>
+    <t>2 Reinf</t>
+  </si>
+  <si>
+    <t>1 GB 2; 1 GB 1 Corps</t>
+  </si>
+  <si>
+    <t>CALCULATE VICTORY: If South Caen or St Lo lost - LOSE GAME.</t>
   </si>
 </sst>
 </file>
@@ -1080,18 +1068,12 @@
                 <c:pt idx="7">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="12">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1107,25 +1089,13 @@
                 <c:pt idx="16">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="17">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="22">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="23">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="24">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2492,7 +2462,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>4</v>
@@ -2552,7 +2522,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>16</v>
@@ -2591,7 +2561,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>16</v>
@@ -2615,7 +2585,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="T3" s="3"/>
     </row>
@@ -2630,7 +2600,7 @@
         <v>2</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>16</v>
@@ -2673,7 +2643,7 @@
         <v>2</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
@@ -2710,7 +2680,7 @@
         <v>2</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
@@ -2747,7 +2717,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>16</v>
@@ -2792,7 +2762,7 @@
         <v>2</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>16</v>
@@ -2825,7 +2795,7 @@
         <v>3</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="4" t="s">
@@ -2858,14 +2828,12 @@
         <v>34</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D10" s="3">
         <v>3</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>132</v>
-      </c>
+      <c r="E10" s="4"/>
       <c r="F10" s="3"/>
       <c r="G10" s="4"/>
       <c r="H10" s="3"/>
@@ -2875,14 +2843,14 @@
       <c r="L10" s="4"/>
       <c r="M10" s="3"/>
       <c r="N10" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T10" s="3"/>
     </row>
@@ -2897,7 +2865,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="4"/>
@@ -2926,13 +2894,13 @@
         <v>39</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D12" s="3">
         <v>1</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>16</v>
@@ -2959,14 +2927,12 @@
         <v>40</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D13" s="3">
         <v>0</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>134</v>
-      </c>
+      <c r="E13" s="4"/>
       <c r="F13" s="3"/>
       <c r="G13" s="4"/>
       <c r="H13" s="3"/>
@@ -2980,7 +2946,7 @@
         <v>21</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q13" s="4" t="s">
         <v>21</v>
@@ -3000,7 +2966,7 @@
         <v>4</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="4" t="s">
@@ -3047,7 +3013,7 @@
         <v>2</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="4"/>
@@ -3078,13 +3044,13 @@
         <v>46</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D16" s="3">
         <v>0</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>16</v>
@@ -3129,7 +3095,7 @@
         <v>2</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
@@ -3170,7 +3136,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>16</v>
@@ -3204,9 +3170,7 @@
       <c r="D19" s="3">
         <v>1</v>
       </c>
-      <c r="E19" s="4" t="s">
-        <v>132</v>
-      </c>
+      <c r="E19" s="4"/>
       <c r="F19" s="3" t="s">
         <v>16</v>
       </c>
@@ -3231,7 +3195,7 @@
         <v>18</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T19" s="3"/>
     </row>
@@ -3272,9 +3236,7 @@
       <c r="D21" s="3">
         <v>2</v>
       </c>
-      <c r="E21" s="4" t="s">
-        <v>132</v>
-      </c>
+      <c r="E21" s="4"/>
       <c r="F21" s="3"/>
       <c r="G21" s="4"/>
       <c r="H21" s="3" t="s">
@@ -3305,7 +3267,7 @@
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="T21" s="3"/>
     </row>
@@ -3320,7 +3282,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="4"/>
@@ -3357,7 +3319,7 @@
         <v>2</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="4"/>
@@ -3389,9 +3351,7 @@
       <c r="D24" s="3">
         <v>0</v>
       </c>
-      <c r="E24" s="4" t="s">
-        <v>140</v>
-      </c>
+      <c r="E24" s="4"/>
       <c r="F24" s="3"/>
       <c r="G24" s="4"/>
       <c r="H24" s="3"/>
@@ -3423,7 +3383,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>16</v>
@@ -3443,7 +3403,7 @@
       <c r="Q25" s="4"/>
       <c r="R25" s="4"/>
       <c r="S25" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="T25" s="3"/>
     </row>
@@ -3457,9 +3417,7 @@
       <c r="D26" s="3">
         <v>1</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>132</v>
-      </c>
+      <c r="E26" s="4"/>
       <c r="F26" s="3"/>
       <c r="G26" s="4"/>
       <c r="H26" s="3"/>
@@ -3485,7 +3443,7 @@
     <row r="27" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B27" s="4"/>
       <c r="C27" s="6" t="s">
-        <v>75</v>
+        <v>137</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="4"/>
@@ -3507,7 +3465,7 @@
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B28" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>74</v>
@@ -3518,7 +3476,7 @@
         <v>16</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H28" s="3"/>
       <c r="I28" s="4"/>
@@ -3536,10 +3494,10 @@
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B29" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="4"/>
@@ -3563,10 +3521,10 @@
     </row>
     <row r="30" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B30" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D30" s="3"/>
       <c r="E30" s="4"/>
@@ -3590,16 +3548,16 @@
       <c r="Q30" s="4"/>
       <c r="R30" s="4"/>
       <c r="S30" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="T30" s="3"/>
     </row>
     <row r="31" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B31" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="4"/>
@@ -3621,10 +3579,10 @@
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B32" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
@@ -3646,10 +3604,10 @@
     </row>
     <row r="33" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B33" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="4"/>
@@ -3671,10 +3629,10 @@
     </row>
     <row r="34" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B34" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="4"/>
@@ -3698,10 +3656,10 @@
     </row>
     <row r="35" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B35" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="4"/>
@@ -3723,10 +3681,10 @@
     </row>
     <row r="36" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B36" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="4"/>
@@ -3752,10 +3710,10 @@
     </row>
     <row r="37" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B37" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="4"/>
@@ -3773,16 +3731,16 @@
       <c r="Q37" s="4"/>
       <c r="R37" s="4"/>
       <c r="S37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="T37" s="3"/>
     </row>
     <row r="38" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B38" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="4"/>
@@ -3804,10 +3762,10 @@
     </row>
     <row r="39" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B39" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="4"/>
@@ -3829,10 +3787,10 @@
     </row>
     <row r="40" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B40" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>96</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="4"/>
@@ -3850,13 +3808,13 @@
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
       <c r="S40" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="T40" s="3"/>
     </row>
     <row r="41" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B41" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>59</v>
@@ -3881,7 +3839,7 @@
     </row>
     <row r="42" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B42" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>59</v>
@@ -3906,7 +3864,7 @@
     </row>
     <row r="43" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B43" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>63</v>
@@ -3933,7 +3891,7 @@
     </row>
     <row r="44" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B44" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
@@ -3956,7 +3914,7 @@
     </row>
     <row r="45" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B45" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
@@ -3979,7 +3937,7 @@
     </row>
     <row r="46" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B46" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
@@ -4002,7 +3960,7 @@
     </row>
     <row r="47" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B47" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
@@ -4025,7 +3983,7 @@
     </row>
     <row r="48" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B48" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
@@ -4048,7 +4006,7 @@
     </row>
     <row r="49" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B49" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
@@ -4071,7 +4029,7 @@
     </row>
     <row r="50" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B50" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>

</xml_diff>